<commit_message>
fixed the outstanding warrants
</commit_message>
<xml_diff>
--- a/2_Funds_parser/Outputs/final_ranking_2025Q4.xlsx
+++ b/2_Funds_parser/Outputs/final_ranking_2025Q4.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="M6 2025Q4 run10" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="M6 2025Q4 run9" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -518,7 +518,7 @@
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>market_cap_usd</t>
+          <t>fully_diluted_market_cap_usd</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
@@ -587,7 +587,7 @@
         <v>0.82</v>
       </c>
       <c r="S2" t="n">
-        <v>1874779361</v>
+        <v>2301149983.406067</v>
       </c>
       <c r="T2" t="n">
         <v>1</v>
@@ -653,7 +653,7 @@
         <v>0.18</v>
       </c>
       <c r="S3" t="n">
-        <v>72121574</v>
+        <v>160800006.3896179</v>
       </c>
       <c r="T3" t="n">
         <v>2</v>
@@ -719,7 +719,7 @@
         <v>0.1</v>
       </c>
       <c r="S4" t="n">
-        <v>243805042</v>
+        <v>271599994.6594238</v>
       </c>
       <c r="T4" t="n">
         <v>1</v>
@@ -785,7 +785,7 @@
         <v>0.95</v>
       </c>
       <c r="S5" t="n">
-        <v>4437085953</v>
+        <v>4523794256.839752</v>
       </c>
       <c r="T5" t="n">
         <v>1</v>
@@ -851,7 +851,7 @@
         <v>0.95</v>
       </c>
       <c r="S6" t="n">
-        <v>314910605</v>
+        <v>358799998.7602234</v>
       </c>
       <c r="T6" t="n">
         <v>1</v>
@@ -917,7 +917,7 @@
         <v>0.13</v>
       </c>
       <c r="S7" t="n">
-        <v>1613916009</v>
+        <v>2622100009.918213</v>
       </c>
       <c r="T7" t="n">
         <v>2</v>
@@ -983,7 +983,7 @@
         <v>0.65</v>
       </c>
       <c r="S8" t="n">
-        <v>2077675978</v>
+        <v>2177950065.612793</v>
       </c>
       <c r="T8" t="n">
         <v>4</v>

</xml_diff>